<commit_message>
fix: restore Excel template formulas
</commit_message>
<xml_diff>
--- a/新收费计划计算.xlsx
+++ b/新收费计划计算.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="利润20%" sheetId="4" r:id="Rb5fefb65ec2b4adf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defer 延付利息（待确认）" sheetId="2" r:id="R267a0d790de24466"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="利润20%" sheetId="4" r:id="R48fae6417f164387"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defer 延付利息（待确认）" sheetId="2" r:id="Ra8649aace58f4c39"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -123,6 +123,9 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">N=MAX(I,E)</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">例子</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Period</x:t>
@@ -1146,54 +1149,135 @@
     <x:row r="3" ht="100" customHeight="1">
       <x:c r="A3" s="41"/>
       <x:c r="B3" s="42"/>
-      <x:c r="C3" s="87"/>
+      <x:c r="C3" s="87" t="s">
+        <x:v>38</x:v>
+      </x:c>
       <x:c r="D3" s="88"/>
       <x:c r="E3" s="89"/>
       <x:c r="F3" s="90"/>
       <x:c r="G3" s="91"/>
       <x:c r="H3" s="92"/>
-      <x:c r="I3" s="93"/>
-      <x:c r="J3" s="93"/>
-      <x:c r="K3" s="50"/>
-      <x:c r="L3" s="94"/>
-      <x:c r="M3" s="95"/>
-      <x:c r="N3" s="95"/>
-      <x:c r="O3" s="96"/>
-      <x:c r="P3" s="94"/>
-      <x:c r="Q3" s="96"/>
-      <x:c r="R3" s="97"/>
-      <x:c r="S3" s="98"/>
-      <x:c r="T3" s="98"/>
-      <x:c r="U3" s="96"/>
-      <x:c r="V3" s="98"/>
-      <x:c r="W3" s="98"/>
+      <x:c r="I3" s="93">
+        <x:v>45658</x:v>
+      </x:c>
+      <x:c r="J3" s="93">
+        <x:v>45747</x:v>
+      </x:c>
+      <x:c r="K3" s="50" t="n">
+        <x:f>J3-I3+1</x:f>
+        <x:v>90</x:v>
+      </x:c>
+      <x:c r="L3" s="94">
+        <x:v>381833.81</x:v>
+      </x:c>
+      <x:c r="M3" s="95">
+        <x:v>32375.84</x:v>
+      </x:c>
+      <x:c r="N3" s="95">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O3" s="96" t="n">
+        <x:f>M3-N3</x:f>
+        <x:v>32375.84</x:v>
+      </x:c>
+      <x:c r="P3" s="94" t="n">
+        <x:f>373455.51+94978.23</x:f>
+        <x:v>468433.74</x:v>
+      </x:c>
+      <x:c r="Q3" s="96" t="n">
+        <x:f>P3-L3-O3</x:f>
+        <x:v>54224.09</x:v>
+      </x:c>
+      <x:c r="R3" s="97" t="n">
+        <x:f>Q3/(L3+O3)</x:f>
+        <x:v>0.1309097699679377</x:v>
+      </x:c>
+      <x:c r="S3" s="98">
+        <x:v>430697.58</x:v>
+      </x:c>
+      <x:c r="T3" s="98" t="n">
+        <x:f>S3+O3</x:f>
+        <x:v>463073.42000000004</x:v>
+      </x:c>
+      <x:c r="U3" s="96" t="n">
+        <x:f>P3-T3</x:f>
+        <x:v>5360.319999999949</x:v>
+      </x:c>
+      <x:c r="V3" s="98" t="n">
+        <x:f>IF(U3&gt;0,U3*0.2,0)</x:f>
+        <x:v>1072.0639999999898</x:v>
+      </x:c>
+      <x:c r="W3" s="98" t="n">
+        <x:f>MAX(T3,P3)</x:f>
+        <x:v>468433.74</x:v>
+      </x:c>
       <x:c r="X3" s="99"/>
       <x:c r="Y3" s="99"/>
     </x:row>
     <x:row r="4" ht="100" customHeight="1">
       <x:c r="A4" s="41"/>
       <x:c r="B4" s="42"/>
-      <x:c r="C4" s="87"/>
+      <x:c r="C4" s="87" t="s">
+        <x:v>38</x:v>
+      </x:c>
       <x:c r="D4" s="88"/>
       <x:c r="E4" s="89"/>
       <x:c r="F4" s="90"/>
       <x:c r="G4" s="91"/>
       <x:c r="H4" s="92"/>
-      <x:c r="I4" s="93"/>
-      <x:c r="J4" s="93"/>
-      <x:c r="K4" s="50"/>
-      <x:c r="L4" s="94"/>
-      <x:c r="M4" s="95"/>
-      <x:c r="N4" s="95"/>
-      <x:c r="O4" s="96"/>
-      <x:c r="P4" s="94"/>
-      <x:c r="Q4" s="96"/>
-      <x:c r="R4" s="97"/>
-      <x:c r="S4" s="98"/>
-      <x:c r="T4" s="98"/>
-      <x:c r="U4" s="96"/>
-      <x:c r="V4" s="98"/>
-      <x:c r="W4" s="98"/>
+      <x:c r="I4" s="93">
+        <x:v>45658</x:v>
+      </x:c>
+      <x:c r="J4" s="93">
+        <x:v>45747</x:v>
+      </x:c>
+      <x:c r="K4" s="50" t="n">
+        <x:f>J4-I4+1</x:f>
+        <x:v>90</x:v>
+      </x:c>
+      <x:c r="L4" s="94">
+        <x:v>1000000</x:v>
+      </x:c>
+      <x:c r="M4" s="95">
+        <x:v>100000</x:v>
+      </x:c>
+      <x:c r="N4" s="95">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O4" s="96" t="n">
+        <x:f>M4-N4</x:f>
+        <x:v>100000</x:v>
+      </x:c>
+      <x:c r="P4" s="94">
+        <x:v>1110000</x:v>
+      </x:c>
+      <x:c r="Q4" s="96" t="n">
+        <x:f>P4-L4-O4</x:f>
+        <x:v>10000</x:v>
+      </x:c>
+      <x:c r="R4" s="97" t="n">
+        <x:f>Q4/(L4+O4)</x:f>
+        <x:v>0.00909090909090909</x:v>
+      </x:c>
+      <x:c r="S4" s="98">
+        <x:v>1000000</x:v>
+      </x:c>
+      <x:c r="T4" s="98" t="n">
+        <x:f>S4+O4</x:f>
+        <x:v>1100000</x:v>
+      </x:c>
+      <x:c r="U4" s="96" t="n">
+        <x:f>P4-T4</x:f>
+        <x:v>10000</x:v>
+      </x:c>
+      <x:c r="V4" s="98" t="n">
+        <x:f>IF(U4&gt;0,U4*0.2,0)</x:f>
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="W4" s="98" t="n">
+        <x:f>MAX(T4,P4)</x:f>
+        <x:v>1110000</x:v>
+      </x:c>
       <x:c r="X4" s="99"/>
       <x:c r="Y4" s="99"/>
     </x:row>
@@ -1232,14 +1316,10 @@
       <x:c r="Q12" s="103"/>
     </x:row>
     <x:row r="8323">
-      <x:c r="AE8323" s="4">
-        <x:v>10767.5</x:v>
-      </x:c>
+      <x:c r="AE8323" s="4"/>
     </x:row>
     <x:row r="8324">
-      <x:c r="AO8324" s="4">
-        <x:v>702</x:v>
-      </x:c>
+      <x:c r="AO8324" s="4"/>
     </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="I3:I4">
@@ -1320,7 +1400,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="I1" s="12" t="s">
-        <x:v>38</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="J1" s="13"/>
       <x:c r="K1" s="14" t="s">
@@ -1354,16 +1434,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="U1" s="20" t="s">
-        <x:v>39</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="V1" s="21" t="s">
-        <x:v>40</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="W1" s="102" t="s">
-        <x:v>41</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="X1" s="23" t="s">
-        <x:v>42</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="Y1" s="22" t="s">
         <x:v>22</x:v>
@@ -1388,7 +1468,7 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="J2" s="32" t="s">
-        <x:v>43</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="K2" s="33" t="s">
         <x:v>25</x:v>
@@ -1409,10 +1489,10 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="Q2" s="35" t="s">
-        <x:v>44</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="R2" s="35" t="s">
-        <x:v>45</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="S2" s="34" t="s">
         <x:v>33</x:v>
@@ -1421,19 +1501,19 @@
         <x:v>34</x:v>
       </x:c>
       <x:c r="U2" s="36" t="s">
-        <x:v>46</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="V2" s="37" t="s">
-        <x:v>47</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="W2" s="38" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="X2" s="39" t="s">
-        <x:v>49</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="Y2" s="40" t="s">
-        <x:v>50</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="Z2" s="26"/>
       <x:c r="AA2" s="26"/>
@@ -1442,7 +1522,7 @@
       <x:c r="A3" s="41"/>
       <x:c r="B3" s="42"/>
       <x:c r="C3" s="43" t="s">
-        <x:v>51</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="D3" s="44"/>
       <x:c r="E3" s="45"/>
@@ -1517,7 +1597,7 @@
       <x:c r="A4" s="41"/>
       <x:c r="B4" s="42"/>
       <x:c r="C4" s="43" t="s">
-        <x:v>52</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="D4" s="44"/>
       <x:c r="E4" s="45"/>
@@ -1592,7 +1672,7 @@
       <x:c r="A5" s="41"/>
       <x:c r="B5" s="42"/>
       <x:c r="C5" s="43" t="s">
-        <x:v>53</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="D5" s="44"/>
       <x:c r="E5" s="45"/>
@@ -1667,7 +1747,7 @@
       <x:c r="A6" s="41"/>
       <x:c r="B6" s="42"/>
       <x:c r="C6" s="43" t="s">
-        <x:v>54</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="D6" s="44"/>
       <x:c r="E6" s="45"/>

</xml_diff>